<commit_message>
Added new RDF data schemes and visual schemes for environment-table04-05, and fixed XLSX spreadsheet for environment-table04
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table04.xlsx
+++ b/sources/table_normalization/xlsx/environment-table04.xlsx
@@ -157,7 +157,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="#,##0.000"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -319,11 +319,24 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
@@ -337,23 +350,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -638,30 +638,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13">
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:13">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="2:13">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="2:13" ht="30" customHeight="1">
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -696,7 +696,7 @@
       </c>
     </row>
     <row r="7" spans="2:13">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -734,38 +734,38 @@
       </c>
     </row>
     <row r="8" spans="2:13" ht="15" customHeight="1">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="8" t="s">
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="2:13" ht="15" customHeight="1">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="9"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="14"/>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" s="16" t="s">
@@ -1034,38 +1034,38 @@
       </c>
     </row>
     <row r="17" spans="2:13" ht="15" customHeight="1">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="8" t="s">
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="15" customHeight="1">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="9"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="14"/>
     </row>
     <row r="19" spans="2:13">
       <c r="B19" s="16" t="s">
@@ -1334,38 +1334,38 @@
       </c>
     </row>
     <row r="26" spans="2:13" ht="15" customHeight="1">
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="8" t="s">
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="27" spans="2:13" ht="15" customHeight="1">
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="9"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="14"/>
     </row>
     <row r="28" spans="2:13">
       <c r="B28" s="16" t="s">
@@ -1672,38 +1672,38 @@
       </c>
     </row>
     <row r="36" spans="2:13" ht="15" customHeight="1">
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7"/>
-      <c r="M36" s="8" t="s">
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="12"/>
+      <c r="L36" s="12"/>
+      <c r="M36" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="37" spans="2:13" ht="15" customHeight="1">
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="9"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="12"/>
+      <c r="M37" s="14"/>
     </row>
     <row r="38" spans="2:13">
       <c r="B38" s="16" t="s">
@@ -2010,38 +2010,38 @@
       </c>
     </row>
     <row r="46" spans="2:13" ht="15" customHeight="1">
-      <c r="B46" s="6" t="s">
+      <c r="B46" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
-      <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
-      <c r="L46" s="7"/>
-      <c r="M46" s="8" t="s">
+      <c r="C46" s="12"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12"/>
+      <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
+      <c r="L46" s="12"/>
+      <c r="M46" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="47" spans="2:13" ht="15" customHeight="1">
-      <c r="B47" s="6" t="s">
+      <c r="B47" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="7"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
-      <c r="L47" s="7"/>
-      <c r="M47" s="9"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="12"/>
+      <c r="J47" s="12"/>
+      <c r="K47" s="12"/>
+      <c r="L47" s="12"/>
+      <c r="M47" s="14"/>
     </row>
     <row r="48" spans="2:13">
       <c r="B48" s="16" t="s">
@@ -2348,38 +2348,38 @@
       </c>
     </row>
     <row r="56" spans="2:13" ht="15" customHeight="1">
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="7"/>
-      <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
-      <c r="H56" s="7"/>
-      <c r="I56" s="7"/>
-      <c r="J56" s="7"/>
-      <c r="K56" s="7"/>
-      <c r="L56" s="7"/>
-      <c r="M56" s="8" t="s">
+      <c r="C56" s="12"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="12"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="12"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="12"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="12"/>
+      <c r="M56" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="57" spans="2:13" ht="15" customHeight="1">
-      <c r="B57" s="6" t="s">
+      <c r="B57" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
-      <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
-      <c r="H57" s="7"/>
-      <c r="I57" s="7"/>
-      <c r="J57" s="7"/>
-      <c r="K57" s="7"/>
-      <c r="L57" s="7"/>
-      <c r="M57" s="9"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="12"/>
+      <c r="J57" s="12"/>
+      <c r="K57" s="12"/>
+      <c r="L57" s="12"/>
+      <c r="M57" s="14"/>
     </row>
     <row r="58" spans="2:13">
       <c r="B58" s="16" t="s">
@@ -2686,38 +2686,38 @@
       </c>
     </row>
     <row r="66" spans="2:13" ht="15" customHeight="1">
-      <c r="B66" s="6" t="s">
+      <c r="B66" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
-      <c r="F66" s="7"/>
-      <c r="G66" s="7"/>
-      <c r="H66" s="7"/>
-      <c r="I66" s="7"/>
-      <c r="J66" s="7"/>
-      <c r="K66" s="7"/>
-      <c r="L66" s="7"/>
-      <c r="M66" s="8" t="s">
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
+      <c r="F66" s="12"/>
+      <c r="G66" s="12"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="12"/>
+      <c r="J66" s="12"/>
+      <c r="K66" s="12"/>
+      <c r="L66" s="12"/>
+      <c r="M66" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="67" spans="2:13" ht="15" customHeight="1">
-      <c r="B67" s="6" t="s">
+      <c r="B67" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7"/>
-      <c r="E67" s="7"/>
-      <c r="F67" s="7"/>
-      <c r="G67" s="7"/>
-      <c r="H67" s="7"/>
-      <c r="I67" s="7"/>
-      <c r="J67" s="7"/>
-      <c r="K67" s="7"/>
-      <c r="L67" s="7"/>
-      <c r="M67" s="9"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12"/>
+      <c r="G67" s="12"/>
+      <c r="H67" s="12"/>
+      <c r="I67" s="12"/>
+      <c r="J67" s="12"/>
+      <c r="K67" s="12"/>
+      <c r="L67" s="12"/>
+      <c r="M67" s="14"/>
     </row>
     <row r="68" spans="2:13">
       <c r="B68" s="16" t="s">
@@ -3024,38 +3024,38 @@
       </c>
     </row>
     <row r="76" spans="2:13" ht="15" customHeight="1">
-      <c r="B76" s="6" t="s">
+      <c r="B76" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C76" s="7"/>
-      <c r="D76" s="7"/>
-      <c r="E76" s="7"/>
-      <c r="F76" s="7"/>
-      <c r="G76" s="7"/>
-      <c r="H76" s="7"/>
-      <c r="I76" s="7"/>
-      <c r="J76" s="7"/>
-      <c r="K76" s="7"/>
-      <c r="L76" s="7"/>
-      <c r="M76" s="8" t="s">
+      <c r="C76" s="12"/>
+      <c r="D76" s="12"/>
+      <c r="E76" s="12"/>
+      <c r="F76" s="12"/>
+      <c r="G76" s="12"/>
+      <c r="H76" s="12"/>
+      <c r="I76" s="12"/>
+      <c r="J76" s="12"/>
+      <c r="K76" s="12"/>
+      <c r="L76" s="12"/>
+      <c r="M76" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="77" spans="2:13" ht="15" customHeight="1">
-      <c r="B77" s="6" t="s">
+      <c r="B77" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C77" s="7"/>
-      <c r="D77" s="7"/>
-      <c r="E77" s="7"/>
-      <c r="F77" s="7"/>
-      <c r="G77" s="7"/>
-      <c r="H77" s="7"/>
-      <c r="I77" s="7"/>
-      <c r="J77" s="7"/>
-      <c r="K77" s="7"/>
-      <c r="L77" s="7"/>
-      <c r="M77" s="9"/>
+      <c r="C77" s="12"/>
+      <c r="D77" s="12"/>
+      <c r="E77" s="12"/>
+      <c r="F77" s="12"/>
+      <c r="G77" s="12"/>
+      <c r="H77" s="12"/>
+      <c r="I77" s="12"/>
+      <c r="J77" s="12"/>
+      <c r="K77" s="12"/>
+      <c r="L77" s="12"/>
+      <c r="M77" s="14"/>
     </row>
     <row r="78" spans="2:13">
       <c r="B78" s="16" t="s">
@@ -3362,38 +3362,38 @@
       </c>
     </row>
     <row r="86" spans="2:13" ht="15" customHeight="1">
-      <c r="B86" s="6" t="s">
+      <c r="B86" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C86" s="7"/>
-      <c r="D86" s="7"/>
-      <c r="E86" s="7"/>
-      <c r="F86" s="7"/>
-      <c r="G86" s="7"/>
-      <c r="H86" s="7"/>
-      <c r="I86" s="7"/>
-      <c r="J86" s="7"/>
-      <c r="K86" s="7"/>
-      <c r="L86" s="7"/>
-      <c r="M86" s="8" t="s">
+      <c r="C86" s="12"/>
+      <c r="D86" s="12"/>
+      <c r="E86" s="12"/>
+      <c r="F86" s="12"/>
+      <c r="G86" s="12"/>
+      <c r="H86" s="12"/>
+      <c r="I86" s="12"/>
+      <c r="J86" s="12"/>
+      <c r="K86" s="12"/>
+      <c r="L86" s="12"/>
+      <c r="M86" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="87" spans="2:13" ht="15" customHeight="1">
-      <c r="B87" s="6" t="s">
+      <c r="B87" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C87" s="7"/>
-      <c r="D87" s="7"/>
-      <c r="E87" s="7"/>
-      <c r="F87" s="7"/>
-      <c r="G87" s="7"/>
-      <c r="H87" s="7"/>
-      <c r="I87" s="7"/>
-      <c r="J87" s="7"/>
-      <c r="K87" s="7"/>
-      <c r="L87" s="7"/>
-      <c r="M87" s="9"/>
+      <c r="C87" s="12"/>
+      <c r="D87" s="12"/>
+      <c r="E87" s="12"/>
+      <c r="F87" s="12"/>
+      <c r="G87" s="12"/>
+      <c r="H87" s="12"/>
+      <c r="I87" s="12"/>
+      <c r="J87" s="12"/>
+      <c r="K87" s="12"/>
+      <c r="L87" s="12"/>
+      <c r="M87" s="14"/>
     </row>
     <row r="88" spans="2:13">
       <c r="B88" s="16" t="s">
@@ -3700,15 +3700,27 @@
       </c>
     </row>
     <row r="97" spans="2:14">
-      <c r="B97" s="12" t="s">
+      <c r="B97" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="N97" s="13" t="s">
+      <c r="N97" s="9" t="s">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B8:L8"/>
+    <mergeCell ref="B9:L9"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="B66:L66"/>
+    <mergeCell ref="B67:L67"/>
+    <mergeCell ref="B26:L26"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B46:L46"/>
     <mergeCell ref="B76:L76"/>
     <mergeCell ref="B77:L77"/>
     <mergeCell ref="B86:L86"/>
@@ -3725,18 +3737,6 @@
     <mergeCell ref="B47:L47"/>
     <mergeCell ref="B56:L56"/>
     <mergeCell ref="B57:L57"/>
-    <mergeCell ref="B66:L66"/>
-    <mergeCell ref="B67:L67"/>
-    <mergeCell ref="B26:L26"/>
-    <mergeCell ref="B27:L27"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B37:L37"/>
-    <mergeCell ref="B46:L46"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B8:L8"/>
-    <mergeCell ref="B9:L9"/>
-    <mergeCell ref="B17:L17"/>
-    <mergeCell ref="B18:L18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B97" r:id="rId1"/>

</xml_diff>